<commit_message>
Update screenshots with actual channel-wise table pages
- Bajaj Allianz: Page 110 (Commission Schedule with channel breakdown)
- Go Digit: Page 141 (Channel-wise commission data)
- ICICI Lombard: Page 280 (Channel-wise commission schedule)
- Care Health: Page 29 (Channel distribution summary)
- Star Health: Page 51 (Distribution channel details)
- Niva Bupa: Page 39 (Channel-wise GDPI data)
- IRDAI Industry: Page 301 (POSP and channel statistics)
- GI Council: Page 17 (Industry channel overview)
</commit_message>
<xml_diff>
--- a/insurance_data/output/insurance_screenshots.xlsx
+++ b/insurance_data/output/insurance_screenshots.xlsx
@@ -8,15 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Bajaj Allianz" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Care Health" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Go Digit" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cbdt Itr" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="GI Council Industry" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="ICICI Lombard" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Go Digit" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ICICI Lombard" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Care Health" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Star Health" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Niva Bupa" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="IRDAI Industry" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Niva Bupa" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Star Health" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="HDFC Ergo" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="GI Council" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +35,9 @@
     <font>
       <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -59,9 +60,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -144,10 +146,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>4</row>
+      <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7620000" cy="10763250"/>
+    <ext cx="9525000" cy="13468350"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -168,16 +170,16 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>4</row>
+      <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7620000" cy="5715000"/>
+    <ext cx="9525000" cy="13468350"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -198,16 +200,16 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>4</row>
+      <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7620000" cy="4705350"/>
+    <ext cx="9525000" cy="13468350"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -228,16 +230,16 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>4</row>
+      <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7620000" cy="10763250"/>
+    <ext cx="9525000" cy="5876925"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -258,16 +260,16 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>4</row>
+      <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7620000" cy="10772775"/>
+    <ext cx="9525000" cy="13468350"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -288,16 +290,16 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>4</row>
+      <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7620000" cy="10782300"/>
+    <ext cx="9525000" cy="13468350"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -318,16 +320,16 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>4</row>
+      <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7620000" cy="9858375"/>
+    <ext cx="9525000" cy="12630150"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -348,76 +350,16 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>4</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="7620000" cy="10096500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
 <file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>4</row>
+      <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7620000" cy="10763250"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>4</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="7620000" cy="10763250"/>
+    <ext cx="9525000" cy="13477875"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -727,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -740,50 +682,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source: Annual-Report-2024-2025.pdf</t>
+          <t>Source PDF: Annual-Report-2024-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Page: 38</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Company: HDFC Ergo</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Source: Sample Data</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Page: N/A</t>
+          <t>Page Number: 110</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Channel-wise Health Insurance Business Table</t>
         </is>
       </c>
     </row>
@@ -799,27 +712,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Company: Care Health</t>
+          <t>Company: Go Digit</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source: Religare-Enterprises-AR-24-25_Web-Upload-Spread-C2C.pdf</t>
+          <t>Source PDF: annual-report-for-fy2024-25-gdgil.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Page: 29</t>
+          <t>Page Number: 141</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Channel-wise Health Insurance Business Table</t>
         </is>
       </c>
     </row>
@@ -835,27 +755,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Company: Go Digit</t>
+          <t>Company: ICICI Lombard</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source: annual-report-for-fy2024-25-gdgil.pdf</t>
+          <t>Source PDF: icici_lombard_ar.pdf.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Page: 35</t>
+          <t>Page Number: 280</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Channel-wise Health Insurance Business Table</t>
         </is>
       </c>
     </row>
@@ -871,27 +798,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Company: Cbdt Itr</t>
+          <t>Company: Care Health</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source: cbdt_itr.pdf</t>
+          <t>Source PDF: Religare-Enterprises-AR-24-25.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Page: 90</t>
+          <t>Page Number: 29</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Channel-wise Health Insurance Business Table</t>
         </is>
       </c>
     </row>
@@ -907,27 +841,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Company: GI Council Industry</t>
+          <t>Company: Star Health</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source: gi_council.pdf.pdf</t>
+          <t>Source PDF: star_health_ar.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Page: 17</t>
+          <t>Page Number: 51</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Channel-wise Health Insurance Business Table</t>
         </is>
       </c>
     </row>
@@ -943,27 +884,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Company: ICICI Lombard</t>
+          <t>Company: Niva Bupa</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source: icici_lombard_nse.pdf</t>
+          <t>Source PDF: niva_drhp.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Page: 60</t>
+          <t>Page Number: 39</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Channel-wise Health Insurance Business Table</t>
         </is>
       </c>
     </row>
@@ -979,7 +927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -992,14 +940,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source: irdai_ar.pdf.pdf</t>
+          <t>Source PDF: irdai_ar.pdf.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Page: 300</t>
+          <t>Page Number: 301</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Channel-wise Health Insurance Business Table</t>
         </is>
       </c>
     </row>
@@ -1015,63 +970,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Company: Niva Bupa</t>
+          <t>Company: GI Council</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source: niva_drhp.pdf</t>
+          <t>Source PDF: gi_council.pdf.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Page: 30</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Company: Star Health</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Source: star_health_ar.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Page: 173</t>
+          <t>Page Number: 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Channel-wise Health Insurance Business Table</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add market analysis with D2C, market size, and digital customer data
New Files:
- insurance_market_analysis.xlsx: Comprehensive market analysis
  - Executive Summary with market size projections
  - D2C/Direct Sale channel breakdown (1.68% online, 23.69% offline)
  - Digital customer statistics (800-850 Mn by FY28)
  - Addressable market opportunity analysis

Updated Screenshots (11 new data pages):
- IRDAI Channel Distribution (Health & General)
- GI Council Market Overview & GDPI Split
- Insurance Market Projections (FY18-FY28)
- Digital Transactors Growth Projection
- SAHI Market & Channel Mix Data

Key Findings:
- Total D2C channel: 25.37% of health insurance
- Health insurance market: INR 1.07 Tn growing to 1.8-2.0 Tn by FY28
- Digital transactors: 500-550 Mn (FY23) to 800-850 Mn (FY28)
- Digital insurance premium growing at 30-35% CAGR
</commit_message>
<xml_diff>
--- a/insurance_data/output/insurance_screenshots.xlsx
+++ b/insurance_data/output/insurance_screenshots.xlsx
@@ -7,14 +7,17 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Bajaj Allianz" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Go Digit" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ICICI Lombard" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Care Health" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Star Health" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Niva Bupa" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="IRDAI Industry" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="GI Council" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="IRDAI Health Channels" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="IRDAI General Channels" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="GI Council Overview" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="GI Council GDPI Split" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="GI Council Growth" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Digital Transactors" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="GDPI Projection" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Health Insurance Growth" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Channel GDPI Split" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="SAHI Projection" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="SAHI Channel Mix" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,9 +38,6 @@
     <font>
       <b val="1"/>
       <sz val="14"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -60,10 +60,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -146,10 +145,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>5</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9525000" cy="13468350"/>
+    <ext cx="8572500" cy="11363325"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -170,16 +169,16 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>5</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9525000" cy="13468350"/>
+    <ext cx="8572500" cy="12115800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -200,16 +199,16 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>5</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9525000" cy="13468350"/>
+    <ext cx="8572500" cy="12115800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -230,16 +229,16 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>5</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9525000" cy="5876925"/>
+    <ext cx="8572500" cy="11363325"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -260,16 +259,16 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>5</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9525000" cy="13468350"/>
+    <ext cx="8562975" cy="12134850"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -290,16 +289,16 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>5</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9525000" cy="13468350"/>
+    <ext cx="8562975" cy="12134850"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -320,16 +319,16 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>5</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9525000" cy="12630150"/>
+    <ext cx="8562975" cy="12134850"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -350,16 +349,106 @@
 </wsDr>
 </file>
 
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="12115800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="12115800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>5</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9525000" cy="13477875"/>
+    <ext cx="8572500" cy="12115800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="12115800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -669,34 +758,78 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Company: Bajaj Allianz</t>
+          <t>IRDAI Health Channels</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source PDF: Annual-Report-2024-2025.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Page Number: 110</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Channel-wise Health Insurance Business Table</t>
+          <t>Source: IRDAI_Channel_Distribution_Health_page306.png</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SAHI Projection</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Source: SAHI_Market_Projection_page38.png</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SAHI Channel Mix</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Source: SAHI_Channel_Mix_page45.png</t>
         </is>
       </c>
     </row>
@@ -712,34 +845,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Company: Go Digit</t>
+          <t>IRDAI General Channels</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source PDF: annual-report-for-fy2024-25-gdgil.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Page Number: 141</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Channel-wise Health Insurance Business Table</t>
+          <t>Source: IRDAI_Channel_Distribution_General_page305.png</t>
         </is>
       </c>
     </row>
@@ -755,34 +874,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Company: ICICI Lombard</t>
+          <t>GI Council Overview</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source PDF: icici_lombard_ar.pdf.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Page Number: 280</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Channel-wise Health Insurance Business Table</t>
+          <t>Source: GI_Council_Market_Overview_page18.png</t>
         </is>
       </c>
     </row>
@@ -798,34 +903,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Company: Care Health</t>
+          <t>GI Council GDPI Split</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source PDF: Religare-Enterprises-AR-24-25.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Page Number: 29</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Channel-wise Health Insurance Business Table</t>
+          <t>Source: GI_Council_Channel_GDPI_page71.png</t>
         </is>
       </c>
     </row>
@@ -841,34 +932,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Company: Star Health</t>
+          <t>GI Council Growth</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source PDF: star_health_ar.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Page Number: 51</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Channel-wise Health Insurance Business Table</t>
+          <t>Source: GI_Council_Channel_Growth_page72.png</t>
         </is>
       </c>
     </row>
@@ -884,34 +961,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Company: Niva Bupa</t>
+          <t>Digital Transactors</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source PDF: niva_drhp.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Page Number: 39</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Channel-wise Health Insurance Business Table</t>
+          <t>Source: Digital_Transactors_Projection_page12.png</t>
         </is>
       </c>
     </row>
@@ -927,34 +990,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Company: IRDAI Industry</t>
+          <t>GDPI Projection</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source PDF: irdai_ar.pdf.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Page Number: 301</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Channel-wise Health Insurance Business Table</t>
+          <t>Source: Insurance_GDPI_Projection_page14.png</t>
         </is>
       </c>
     </row>
@@ -970,34 +1019,49 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Company: GI Council</t>
+          <t>Health Insurance Growth</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source PDF: gi_council.pdf.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Page Number: 17</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Channel-wise Health Insurance Business Table</t>
+          <t>Source: Health_Insurance_Growth_page18.png</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Channel GDPI Split</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Source: Channel_GDPI_Split_page26.png</t>
         </is>
       </c>
     </row>

</xml_diff>